<commit_message>
Plantilla de carga: ejemplos de los 3 tipos + hoja de instrucciones
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantilla_carga_preguntas.xlsx
+++ b/docs/plantilla_carga_preguntas.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="preguntas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,14 +428,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
@@ -429,52 +444,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>seccion</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>tipo_pregunta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>pregunta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>opcion_1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>opcion_2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>opcion_3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>opcion_4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>opcion_correcta</t>
         </is>
@@ -489,7 +504,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -517,7 +532,11 @@
           <t>Londres</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
       <c r="J2" t="n">
         <v>2</v>
       </c>
@@ -531,7 +550,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Conocimiento</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -541,7 +560,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>¿2+2?</t>
+          <t>¿Cuánto es 2 + 2?</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -559,11 +578,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
         <v>2</v>
       </c>
@@ -596,17 +611,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Opción A</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Opción B</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Opción C</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -668,19 +683,229 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>opcion_opinion</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>¿Cómo calificaría la organización?</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mala</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bienestar Docente</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Encuesta</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>abierta</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>¿Qué temas reforzaría?</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>¿Qué temas le gustaría reforzar?</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Columna</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nombre del evento. Debe existir previamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nombre del grupo (opcional). Vacío = sección COMÚN del evento (todos los grupos la ven). Con valor = sección específica de ese grupo (debe existir en el evento).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>seccion</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nombre de la sección. Se crea si no existe (con el alcance según 'grupo').</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tipo_pregunta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Uno de: opcion_unica | abierta | opcion_opinion</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pregunta</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Texto/enunciado de la pregunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>opcion_1..opcion_4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Textos de las opciones. Llenar de izquierda a derecha. Vacío en 'abierta'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>opcion_correcta</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Número (1-4) de la opción correcta. SOLO para 'opcion_unica'. Vacío en 'abierta' y 'opcion_opinion'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Comportamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>opcion_unica</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Opción múltiple con UNA respuesta correcta. Puntúa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>opcion_opinion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Opciones de opinión/encuesta. Cualquiera es válida, NO puntúa, pero se registra la elegida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>abierta</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Respuesta de texto libre. Sin opciones, NO puntúa.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>